<commit_message>
update reg files to working model
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\simpaths_dev\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F518E279-5FED-44B4-840A-F9BBB1EBFF47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA49ECF-19B1-4886-A4E2-E700B2D0809E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="23520" windowHeight="12315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -546,7 +546,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>4.1855465085565644</v>
+        <v>4.1711681750766845</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -554,7 +554,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>7.4908409588260065</v>
+        <v>7.4721811659270996</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -562,7 +562,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>6.5883330217266201</v>
+        <v>6.5873304709614393</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -570,7 +570,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>1.8161778493855598</v>
+        <v>1.8134869481636644</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
switch self-rated health to MCS and PCS in social care and partnership
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\simpaths_dev\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA49ECF-19B1-4886-A4E2-E700B2D0809E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1C3B384-2AC4-4E96-ADA1-E5A82DDD087B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="23520" windowHeight="12315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="648" windowWidth="23232" windowHeight="12312" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -514,7 +514,7 @@
         <v>6</v>
       </c>
       <c r="B9">
-        <v>1.036047441983782</v>
+        <v>1.0378978412687669</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -522,7 +522,7 @@
         <v>7</v>
       </c>
       <c r="B10">
-        <v>0.84870070750541715</v>
+        <v>0.85083051214205796</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update housing and mortgage wealth parameters
</commit_message>
<xml_diff>
--- a/input/reg_RMSE.xlsx
+++ b/input/reg_RMSE.xlsx
@@ -1,148 +1,132 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFiles\99 DEV ENV\JAS-MINE\SimPaths\input\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7296AE34-F10A-4EE7-85E3-28BED895BB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheets>
-    <sheet name="UK" sheetId="1" r:id="rId1"/>
+    <sheet name="UK" sheetId="1" r:id="R8e47c9e760174206"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
-  <si>
-    <t>REGRESSOR</t>
-  </si>
-  <si>
-    <t>COEFFICIENT</t>
-  </si>
-  <si>
-    <t>W1fa</t>
-  </si>
-  <si>
-    <t>W1ma</t>
-  </si>
-  <si>
-    <t>W1fb</t>
-  </si>
-  <si>
-    <t>W1mb</t>
-  </si>
-  <si>
-    <t>I1b</t>
-  </si>
-  <si>
-    <t>I2b</t>
-  </si>
-  <si>
-    <t>I3b</t>
-  </si>
-  <si>
-    <t>S2d</t>
-  </si>
-  <si>
-    <t>S2e</t>
-  </si>
-  <si>
-    <t>S3c</t>
-  </si>
-  <si>
-    <t>S3d</t>
-  </si>
-  <si>
-    <t>HM1_L</t>
-  </si>
-  <si>
-    <t>HM2_Females_L</t>
-  </si>
-  <si>
-    <t>HM2_Males_L</t>
-  </si>
-  <si>
-    <t>HM2_Females_C</t>
-  </si>
-  <si>
-    <t>HM2_Males_C</t>
-  </si>
-  <si>
-    <t>DHE_MCS1</t>
-  </si>
-  <si>
-    <t>DHE_MCS2_Females</t>
-  </si>
-  <si>
-    <t>DHE_MCS2_Males</t>
-  </si>
-  <si>
-    <t>DHE_PCS1</t>
-  </si>
-  <si>
-    <t>DHE_PCS2_Females</t>
-  </si>
-  <si>
-    <t>DHE_PCS2_Males</t>
-  </si>
-  <si>
-    <t>DLS1</t>
-  </si>
-  <si>
-    <t>DLS2_Females</t>
-  </si>
-  <si>
-    <t>DLS2_Males</t>
-  </si>
-  <si>
-    <t>PW1d</t>
-  </si>
-  <si>
-    <t>PW1f</t>
-  </si>
-  <si>
-    <t>PW2c</t>
-  </si>
-  <si>
-    <t>FW1a</t>
-  </si>
-  <si>
-    <t>HW1c</t>
-  </si>
-  <si>
-    <t>HW1d</t>
-  </si>
-  <si>
-    <t>HW2c</t>
-  </si>
-  <si>
-    <t>HW2d</t>
-  </si>
-  <si>
-    <t>FW2c</t>
-  </si>
-  <si>
-    <t>FW2d</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <si>
+    <t xml:space="preserve">REGRESSOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COEFFICIENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W1fa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W1ma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W1fb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W1mb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I2b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S3d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HM1_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HM2_Females_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HM2_Males_L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HM2_Females_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HM2_Males_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_MCS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_MCS2_Females</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_MCS2_Males</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_PCS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_PCS2_Females</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHE_PCS2_Males</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLS2_Females</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DLS2_Males</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PW1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PW1f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PW2c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FW1a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FW2c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FW2d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HW1c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HW1d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HW2c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HW2d</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -157,13 +141,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -172,23 +150,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -281,7 +249,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -324,25 +292,23 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="38.1796875" customWidth="1"/>
+    <col min="1" max="1" width="38.1640625" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -350,7 +316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -358,7 +324,7 @@
         <v>0.81845421244698169</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -366,7 +332,7 @@
         <v>0.8318231278642283</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -374,7 +340,7 @@
         <v>0.52842580917125537</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -382,7 +348,7 @@
         <v>0.63796656252519179</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -390,7 +356,7 @@
         <v>1.745511065607195</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -398,7 +364,7 @@
         <v>0.97409509625211432</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -406,7 +372,7 @@
         <v>1.1365855588198841</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -414,7 +380,7 @@
         <v>1.036047441983782</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -422,7 +388,7 @@
         <v>0.84870070750541715</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -430,7 +396,7 @@
         <v>1.1484500852818149</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -438,7 +404,7 @@
         <v>1.1927903832324711</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -446,7 +412,7 @@
         <v>4.4608727317206842</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -454,7 +420,7 @@
         <v>4.2488100047405588</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -462,7 +428,7 @@
         <v>3.7376343170238648</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -470,7 +436,7 @@
         <v>2.596866413019931</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -478,7 +444,7 @@
         <v>2.188554316479709</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -486,7 +452,7 @@
         <v>7.966919324090096</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -494,7 +460,7 @@
         <v>7.1657841258237269</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -502,7 +468,7 @@
         <v>6.4859586641425091</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -510,7 +476,7 @@
         <v>7.0661394726712041</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -518,7 +484,7 @@
         <v>6.0523880929117633</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -526,7 +492,7 @@
         <v>5.4222029042219946</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -534,7 +500,7 @@
         <v>1.902513219539105</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -542,7 +508,7 @@
         <v>1.713488168011807</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -550,7 +516,7 @@
         <v>1.6261256004830791</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -558,7 +524,7 @@
         <v>0.98090109999999997</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -566,7 +532,7 @@
         <v>0.77345540000000002</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -574,7 +540,7 @@
         <v>1.0740229999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -582,49 +548,49 @@
         <v>0.50560000000000005</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B31">
         <v>1.2534000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32">
       <c r="A32" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B32">
         <v>0.93769999999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33">
-        <v>0.95802536417754225</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0.20845521180740498</v>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B34">
         <v>0.55981284625299998</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B35">
-        <v>0.41646133070000002</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+        <v>0.1047875817948884</v>
+      </c>
+    </row>
+    <row r="36">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B36">
         <v>0.80487359000000003</v>

</xml_diff>